<commit_message>
added STS dx cat fields
</commit_message>
<xml_diff>
--- a/src/integration_mapping_dict.xlsx
+++ b/src/integration_mapping_dict.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10920"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bullenca/Work/CCDIDC/CCDIDC-2661/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bullenca/Work/Repos/ChildhoodCancerDataInitiative-MCI_JSON2TSV/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2217D66-05A0-9D47-85C1-E6F60FA766E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC43AE6C-7A39-A041-92E2-4276B2E8DB05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34620" yWindow="-5300" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="integration_mapping_dict" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">integration_mapping_dict!$A$1:$H$1088</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">integration_mapping_dict!$A$1:$H$1091</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5424" uniqueCount="1387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5439" uniqueCount="1390">
   <si>
     <t>type</t>
   </si>
@@ -4197,6 +4197,15 @@
   </si>
   <si>
     <t>Archer Fusion Summary</t>
+  </si>
+  <si>
+    <t>DIAGNOSIS_DETAIL_STS.STSDXTP</t>
+  </si>
+  <si>
+    <t>DIAGNOSIS_DETAIL_STS.MH_MHSCAT_STSDXINTGRT_RMS</t>
+  </si>
+  <si>
+    <t>DIAGNOSIS_DETAIL_STS.MH_MHSCAT_STSDXINTGRT_NRSTS</t>
   </si>
 </sst>
 </file>
@@ -4621,7 +4630,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I1088"/>
+  <dimension ref="A1:I1091"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.6640625" customWidth="1"/>
@@ -25536,55 +25545,64 @@
     </row>
     <row r="994" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A994" t="s">
-        <v>1035</v>
+        <v>8</v>
       </c>
       <c r="B994" t="s">
-        <v>1037</v>
+        <v>8</v>
       </c>
       <c r="C994" t="s">
-        <v>1000</v>
+        <v>1387</v>
       </c>
       <c r="D994" t="s">
-        <v>10</v>
-      </c>
-      <c r="G994" s="11">
-        <v>1</v>
+        <v>739</v>
+      </c>
+      <c r="F994">
+        <v>54</v>
+      </c>
+      <c r="H994" t="s">
+        <v>740</v>
       </c>
       <c r="I994" s="1"/>
     </row>
     <row r="995" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A995" t="s">
-        <v>1035</v>
+        <v>8</v>
       </c>
       <c r="B995" t="s">
-        <v>1037</v>
+        <v>8</v>
       </c>
       <c r="C995" t="s">
-        <v>1001</v>
+        <v>1388</v>
       </c>
       <c r="D995" t="s">
-        <v>1038</v>
-      </c>
-      <c r="G995" s="11">
-        <v>2</v>
+        <v>742</v>
+      </c>
+      <c r="F995">
+        <v>55</v>
+      </c>
+      <c r="H995" t="s">
+        <v>740</v>
       </c>
       <c r="I995" s="1"/>
     </row>
     <row r="996" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A996" t="s">
-        <v>1035</v>
+        <v>8</v>
       </c>
       <c r="B996" t="s">
-        <v>1037</v>
+        <v>8</v>
       </c>
       <c r="C996" t="s">
-        <v>1003</v>
+        <v>1389</v>
       </c>
       <c r="D996" t="s">
-        <v>1039</v>
-      </c>
-      <c r="G996" s="11">
-        <v>3</v>
+        <v>742</v>
+      </c>
+      <c r="F996">
+        <v>55</v>
+      </c>
+      <c r="H996" t="s">
+        <v>740</v>
       </c>
       <c r="I996" s="1"/>
     </row>
@@ -25596,13 +25614,13 @@
         <v>1037</v>
       </c>
       <c r="C997" t="s">
-        <v>1005</v>
+        <v>1000</v>
       </c>
       <c r="D997" t="s">
-        <v>1040</v>
+        <v>10</v>
       </c>
       <c r="G997" s="11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I997" s="1"/>
     </row>
@@ -25614,14 +25632,15 @@
         <v>1037</v>
       </c>
       <c r="C998" t="s">
-        <v>1111</v>
+        <v>1001</v>
       </c>
       <c r="D998" t="s">
-        <v>1113</v>
+        <v>1038</v>
       </c>
       <c r="G998" s="11">
-        <v>5</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="I998" s="1"/>
     </row>
     <row r="999" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A999" t="s">
@@ -25631,14 +25650,15 @@
         <v>1037</v>
       </c>
       <c r="C999" t="s">
-        <v>999</v>
+        <v>1003</v>
       </c>
       <c r="D999" t="s">
-        <v>1386</v>
+        <v>1039</v>
       </c>
       <c r="G999" s="11">
-        <v>6</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="I999" s="1"/>
     </row>
     <row r="1000" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1000" t="s">
@@ -25648,17 +25668,15 @@
         <v>1037</v>
       </c>
       <c r="C1000" t="s">
-        <v>1049</v>
+        <v>1005</v>
       </c>
       <c r="D1000" t="s">
-        <v>1050</v>
-      </c>
-      <c r="E1000" t="s">
-        <v>86</v>
+        <v>1040</v>
       </c>
       <c r="G1000" s="11">
-        <v>7</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="I1000" s="1"/>
     </row>
     <row r="1001" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1001" t="s">
@@ -25668,16 +25686,13 @@
         <v>1037</v>
       </c>
       <c r="C1001" t="s">
-        <v>1051</v>
+        <v>1111</v>
       </c>
       <c r="D1001" t="s">
-        <v>1052</v>
-      </c>
-      <c r="E1001" t="s">
-        <v>86</v>
+        <v>1113</v>
       </c>
       <c r="G1001" s="11">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1002" spans="1:9" x14ac:dyDescent="0.2">
@@ -25688,16 +25703,13 @@
         <v>1037</v>
       </c>
       <c r="C1002" t="s">
-        <v>1053</v>
+        <v>999</v>
       </c>
       <c r="D1002" t="s">
-        <v>1054</v>
-      </c>
-      <c r="E1002" t="s">
-        <v>86</v>
+        <v>1386</v>
       </c>
       <c r="G1002" s="11">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="1003" spans="1:9" x14ac:dyDescent="0.2">
@@ -25708,16 +25720,16 @@
         <v>1037</v>
       </c>
       <c r="C1003" t="s">
-        <v>1055</v>
+        <v>1049</v>
       </c>
       <c r="D1003" t="s">
-        <v>1056</v>
+        <v>1050</v>
       </c>
       <c r="E1003" t="s">
         <v>86</v>
       </c>
       <c r="G1003" s="11">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="1004" spans="1:9" x14ac:dyDescent="0.2">
@@ -25728,16 +25740,16 @@
         <v>1037</v>
       </c>
       <c r="C1004" t="s">
-        <v>1057</v>
+        <v>1051</v>
       </c>
       <c r="D1004" t="s">
-        <v>1058</v>
+        <v>1052</v>
       </c>
       <c r="E1004" t="s">
         <v>86</v>
       </c>
       <c r="G1004" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="1005" spans="1:9" x14ac:dyDescent="0.2">
@@ -25748,16 +25760,16 @@
         <v>1037</v>
       </c>
       <c r="C1005" t="s">
-        <v>1059</v>
+        <v>1053</v>
       </c>
       <c r="D1005" t="s">
-        <v>1060</v>
+        <v>1054</v>
       </c>
       <c r="E1005" t="s">
         <v>86</v>
       </c>
       <c r="G1005" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="1006" spans="1:9" x14ac:dyDescent="0.2">
@@ -25768,16 +25780,16 @@
         <v>1037</v>
       </c>
       <c r="C1006" t="s">
-        <v>1061</v>
+        <v>1055</v>
       </c>
       <c r="D1006" t="s">
-        <v>1062</v>
+        <v>1056</v>
       </c>
       <c r="E1006" t="s">
         <v>86</v>
       </c>
       <c r="G1006" s="11">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="1007" spans="1:9" x14ac:dyDescent="0.2">
@@ -25788,16 +25800,16 @@
         <v>1037</v>
       </c>
       <c r="C1007" t="s">
-        <v>1063</v>
+        <v>1057</v>
       </c>
       <c r="D1007" t="s">
-        <v>1064</v>
+        <v>1058</v>
       </c>
       <c r="E1007" t="s">
         <v>86</v>
       </c>
       <c r="G1007" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="1008" spans="1:9" x14ac:dyDescent="0.2">
@@ -25808,16 +25820,16 @@
         <v>1037</v>
       </c>
       <c r="C1008" t="s">
-        <v>1065</v>
+        <v>1059</v>
       </c>
       <c r="D1008" t="s">
-        <v>1066</v>
+        <v>1060</v>
       </c>
       <c r="E1008" t="s">
         <v>86</v>
       </c>
       <c r="G1008" s="11">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1009" spans="1:7" x14ac:dyDescent="0.2">
@@ -25828,16 +25840,16 @@
         <v>1037</v>
       </c>
       <c r="C1009" t="s">
-        <v>1067</v>
+        <v>1061</v>
       </c>
       <c r="D1009" t="s">
-        <v>1068</v>
+        <v>1062</v>
       </c>
       <c r="E1009" t="s">
         <v>86</v>
       </c>
       <c r="G1009" s="11">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="1010" spans="1:7" x14ac:dyDescent="0.2">
@@ -25848,16 +25860,16 @@
         <v>1037</v>
       </c>
       <c r="C1010" t="s">
-        <v>1069</v>
+        <v>1063</v>
       </c>
       <c r="D1010" t="s">
-        <v>1070</v>
+        <v>1064</v>
       </c>
       <c r="E1010" t="s">
         <v>86</v>
       </c>
       <c r="G1010" s="11">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="1011" spans="1:7" x14ac:dyDescent="0.2">
@@ -25868,16 +25880,16 @@
         <v>1037</v>
       </c>
       <c r="C1011" t="s">
-        <v>1071</v>
+        <v>1065</v>
       </c>
       <c r="D1011" t="s">
-        <v>1072</v>
+        <v>1066</v>
       </c>
       <c r="E1011" t="s">
         <v>86</v>
       </c>
       <c r="G1011" s="11">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="1012" spans="1:7" x14ac:dyDescent="0.2">
@@ -25888,16 +25900,16 @@
         <v>1037</v>
       </c>
       <c r="C1012" t="s">
-        <v>1073</v>
+        <v>1067</v>
       </c>
       <c r="D1012" t="s">
-        <v>1074</v>
+        <v>1068</v>
       </c>
       <c r="E1012" t="s">
         <v>86</v>
       </c>
       <c r="G1012" s="11">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="1013" spans="1:7" x14ac:dyDescent="0.2">
@@ -25905,16 +25917,19 @@
         <v>1035</v>
       </c>
       <c r="B1013" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="C1013" t="s">
-        <v>1000</v>
+        <v>1069</v>
       </c>
       <c r="D1013" t="s">
-        <v>10</v>
+        <v>1070</v>
+      </c>
+      <c r="E1013" t="s">
+        <v>86</v>
       </c>
       <c r="G1013" s="11">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="1014" spans="1:7" x14ac:dyDescent="0.2">
@@ -25922,16 +25937,19 @@
         <v>1035</v>
       </c>
       <c r="B1014" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="C1014" t="s">
-        <v>1001</v>
+        <v>1071</v>
       </c>
       <c r="D1014" t="s">
-        <v>1038</v>
+        <v>1072</v>
+      </c>
+      <c r="E1014" t="s">
+        <v>86</v>
       </c>
       <c r="G1014" s="11">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="1015" spans="1:7" x14ac:dyDescent="0.2">
@@ -25939,16 +25957,19 @@
         <v>1035</v>
       </c>
       <c r="B1015" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="C1015" t="s">
-        <v>1003</v>
+        <v>1073</v>
       </c>
       <c r="D1015" t="s">
-        <v>1039</v>
+        <v>1074</v>
+      </c>
+      <c r="E1015" t="s">
+        <v>86</v>
       </c>
       <c r="G1015" s="11">
-        <v>3</v>
+        <v>19</v>
       </c>
     </row>
     <row r="1016" spans="1:7" x14ac:dyDescent="0.2">
@@ -25959,13 +25980,13 @@
         <v>1036</v>
       </c>
       <c r="C1016" t="s">
-        <v>1005</v>
+        <v>1000</v>
       </c>
       <c r="D1016" t="s">
-        <v>1040</v>
+        <v>10</v>
       </c>
       <c r="G1016" s="11">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1017" spans="1:7" x14ac:dyDescent="0.2">
@@ -25976,13 +25997,13 @@
         <v>1036</v>
       </c>
       <c r="C1017" t="s">
-        <v>1111</v>
+        <v>1001</v>
       </c>
       <c r="D1017" t="s">
-        <v>1113</v>
+        <v>1038</v>
       </c>
       <c r="G1017" s="11">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1018" spans="1:7" x14ac:dyDescent="0.2">
@@ -25993,13 +26014,13 @@
         <v>1036</v>
       </c>
       <c r="C1018" t="s">
-        <v>999</v>
+        <v>1003</v>
       </c>
       <c r="D1018" t="s">
-        <v>1386</v>
+        <v>1039</v>
       </c>
       <c r="G1018" s="11">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1019" spans="1:7" x14ac:dyDescent="0.2">
@@ -26010,16 +26031,13 @@
         <v>1036</v>
       </c>
       <c r="C1019" t="s">
-        <v>1018</v>
+        <v>1005</v>
       </c>
       <c r="D1019" t="s">
-        <v>1075</v>
-      </c>
-      <c r="E1019" t="s">
-        <v>86</v>
+        <v>1040</v>
       </c>
       <c r="G1019" s="11">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="1020" spans="1:7" x14ac:dyDescent="0.2">
@@ -26030,16 +26048,13 @@
         <v>1036</v>
       </c>
       <c r="C1020" t="s">
-        <v>1076</v>
+        <v>1111</v>
       </c>
       <c r="D1020" t="s">
-        <v>1077</v>
-      </c>
-      <c r="E1020" t="s">
-        <v>86</v>
+        <v>1113</v>
       </c>
       <c r="G1020" s="11">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1021" spans="1:7" x14ac:dyDescent="0.2">
@@ -26050,16 +26065,13 @@
         <v>1036</v>
       </c>
       <c r="C1021" t="s">
-        <v>1078</v>
+        <v>999</v>
       </c>
       <c r="D1021" t="s">
-        <v>1079</v>
-      </c>
-      <c r="E1021" t="s">
-        <v>86</v>
+        <v>1386</v>
       </c>
       <c r="G1021" s="11">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="1022" spans="1:7" x14ac:dyDescent="0.2">
@@ -26070,16 +26082,16 @@
         <v>1036</v>
       </c>
       <c r="C1022" t="s">
-        <v>1080</v>
+        <v>1018</v>
       </c>
       <c r="D1022" t="s">
-        <v>1081</v>
+        <v>1075</v>
       </c>
       <c r="E1022" t="s">
         <v>86</v>
       </c>
       <c r="G1022" s="11">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="1023" spans="1:7" x14ac:dyDescent="0.2">
@@ -26090,16 +26102,16 @@
         <v>1036</v>
       </c>
       <c r="C1023" t="s">
-        <v>1082</v>
+        <v>1076</v>
       </c>
       <c r="D1023" t="s">
-        <v>1083</v>
+        <v>1077</v>
       </c>
       <c r="E1023" t="s">
         <v>86</v>
       </c>
       <c r="G1023" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="1024" spans="1:7" x14ac:dyDescent="0.2">
@@ -26110,16 +26122,16 @@
         <v>1036</v>
       </c>
       <c r="C1024" t="s">
-        <v>1084</v>
+        <v>1078</v>
       </c>
       <c r="D1024" t="s">
-        <v>1085</v>
+        <v>1079</v>
       </c>
       <c r="E1024" t="s">
         <v>86</v>
       </c>
       <c r="G1024" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="1025" spans="1:8" x14ac:dyDescent="0.2">
@@ -26130,16 +26142,16 @@
         <v>1036</v>
       </c>
       <c r="C1025" t="s">
-        <v>1086</v>
+        <v>1080</v>
       </c>
       <c r="D1025" t="s">
-        <v>1087</v>
+        <v>1081</v>
       </c>
       <c r="E1025" t="s">
         <v>86</v>
       </c>
       <c r="G1025" s="11">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="1026" spans="1:8" x14ac:dyDescent="0.2">
@@ -26150,16 +26162,16 @@
         <v>1036</v>
       </c>
       <c r="C1026" t="s">
-        <v>1071</v>
+        <v>1082</v>
       </c>
       <c r="D1026" t="s">
-        <v>1088</v>
+        <v>1083</v>
       </c>
       <c r="E1026" t="s">
         <v>86</v>
       </c>
       <c r="G1026" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="1027" spans="1:8" x14ac:dyDescent="0.2">
@@ -26170,85 +26182,76 @@
         <v>1036</v>
       </c>
       <c r="C1027" t="s">
-        <v>1073</v>
+        <v>1084</v>
       </c>
       <c r="D1027" t="s">
-        <v>1089</v>
+        <v>1085</v>
       </c>
       <c r="E1027" t="s">
         <v>86</v>
       </c>
       <c r="G1027" s="11">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1028" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1028" t="s">
-        <v>998</v>
+        <v>1035</v>
       </c>
       <c r="B1028" t="s">
-        <v>999</v>
+        <v>1036</v>
       </c>
       <c r="C1028" t="s">
-        <v>1007</v>
+        <v>1086</v>
       </c>
       <c r="D1028" t="s">
-        <v>1008</v>
-      </c>
-      <c r="F1028" s="11">
-        <v>56</v>
-      </c>
-      <c r="G1028" s="9">
-        <v>5</v>
-      </c>
-      <c r="H1028" t="s">
-        <v>152</v>
+        <v>1087</v>
+      </c>
+      <c r="E1028" t="s">
+        <v>86</v>
+      </c>
+      <c r="G1028" s="11">
+        <v>13</v>
       </c>
     </row>
     <row r="1029" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1029" t="s">
-        <v>998</v>
+        <v>1035</v>
       </c>
       <c r="B1029" t="s">
-        <v>999</v>
+        <v>1036</v>
       </c>
       <c r="C1029" t="s">
-        <v>1009</v>
+        <v>1071</v>
       </c>
       <c r="D1029" t="s">
-        <v>1010</v>
-      </c>
-      <c r="F1029" s="11">
-        <v>57</v>
-      </c>
-      <c r="G1029" s="9">
-        <v>6</v>
-      </c>
-      <c r="H1029" t="s">
-        <v>152</v>
+        <v>1088</v>
+      </c>
+      <c r="E1029" t="s">
+        <v>86</v>
+      </c>
+      <c r="G1029" s="11">
+        <v>14</v>
       </c>
     </row>
     <row r="1030" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1030" t="s">
-        <v>998</v>
+        <v>1035</v>
       </c>
       <c r="B1030" t="s">
-        <v>999</v>
+        <v>1036</v>
       </c>
       <c r="C1030" t="s">
-        <v>1011</v>
+        <v>1073</v>
       </c>
       <c r="D1030" t="s">
-        <v>1012</v>
-      </c>
-      <c r="F1030" s="11">
-        <v>58</v>
-      </c>
-      <c r="G1030" s="9">
-        <v>7</v>
-      </c>
-      <c r="H1030" t="s">
-        <v>152</v>
+        <v>1089</v>
+      </c>
+      <c r="E1030" t="s">
+        <v>86</v>
+      </c>
+      <c r="G1030" s="11">
+        <v>15</v>
       </c>
     </row>
     <row r="1031" spans="1:8" x14ac:dyDescent="0.2">
@@ -26259,19 +26262,22 @@
         <v>999</v>
       </c>
       <c r="C1031" t="s">
-        <v>1000</v>
+        <v>1007</v>
       </c>
       <c r="D1031" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1031" s="11">
-        <v>1</v>
+        <v>1008</v>
+      </c>
+      <c r="F1031" s="11">
+        <v>56</v>
+      </c>
+      <c r="G1031" s="9">
+        <v>5</v>
       </c>
       <c r="H1031" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="1032" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="1032" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1032" t="s">
         <v>998</v>
       </c>
@@ -26279,17 +26285,22 @@
         <v>999</v>
       </c>
       <c r="C1032" t="s">
-        <v>1001</v>
+        <v>1009</v>
       </c>
       <c r="D1032" t="s">
-        <v>1002</v>
-      </c>
-      <c r="G1032" s="11">
-        <v>2</v>
-      </c>
-      <c r="H1032" s="12"/>
-    </row>
-    <row r="1033" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+        <v>1010</v>
+      </c>
+      <c r="F1032" s="11">
+        <v>57</v>
+      </c>
+      <c r="G1032" s="9">
+        <v>6</v>
+      </c>
+      <c r="H1032" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="1033" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1033" t="s">
         <v>998</v>
       </c>
@@ -26297,17 +26308,22 @@
         <v>999</v>
       </c>
       <c r="C1033" t="s">
-        <v>1003</v>
+        <v>1011</v>
       </c>
       <c r="D1033" t="s">
-        <v>1004</v>
-      </c>
-      <c r="G1033" s="11">
-        <v>3</v>
-      </c>
-      <c r="H1033" s="12"/>
-    </row>
-    <row r="1034" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+        <v>1012</v>
+      </c>
+      <c r="F1033" s="11">
+        <v>58</v>
+      </c>
+      <c r="G1033" s="9">
+        <v>7</v>
+      </c>
+      <c r="H1033" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1034" t="s">
         <v>998</v>
       </c>
@@ -26315,66 +26331,71 @@
         <v>999</v>
       </c>
       <c r="C1034" t="s">
+        <v>1000</v>
+      </c>
+      <c r="D1034" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1034" s="11">
+        <v>1</v>
+      </c>
+      <c r="H1034" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="1035" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1035" t="s">
+        <v>998</v>
+      </c>
+      <c r="B1035" t="s">
+        <v>999</v>
+      </c>
+      <c r="C1035" t="s">
+        <v>1001</v>
+      </c>
+      <c r="D1035" t="s">
+        <v>1002</v>
+      </c>
+      <c r="G1035" s="11">
+        <v>2</v>
+      </c>
+      <c r="H1035" s="12"/>
+    </row>
+    <row r="1036" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1036" t="s">
+        <v>998</v>
+      </c>
+      <c r="B1036" t="s">
+        <v>999</v>
+      </c>
+      <c r="C1036" t="s">
+        <v>1003</v>
+      </c>
+      <c r="D1036" t="s">
+        <v>1004</v>
+      </c>
+      <c r="G1036" s="11">
+        <v>3</v>
+      </c>
+      <c r="H1036" s="12"/>
+    </row>
+    <row r="1037" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1037" t="s">
+        <v>998</v>
+      </c>
+      <c r="B1037" t="s">
+        <v>999</v>
+      </c>
+      <c r="C1037" t="s">
         <v>1005</v>
       </c>
-      <c r="D1034" t="s">
+      <c r="D1037" t="s">
         <v>1006</v>
       </c>
-      <c r="G1034" s="11">
+      <c r="G1037" s="11">
         <v>4</v>
       </c>
-      <c r="H1034" s="12"/>
-    </row>
-    <row r="1035" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1035" t="s">
-        <v>1013</v>
-      </c>
-      <c r="B1035" t="s">
-        <v>1033</v>
-      </c>
-      <c r="C1035" t="s">
-        <v>1000</v>
-      </c>
-      <c r="D1035" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1035" s="11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="1036" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1036" t="s">
-        <v>1013</v>
-      </c>
-      <c r="B1036" t="s">
-        <v>1033</v>
-      </c>
-      <c r="C1036" t="s">
-        <v>1001</v>
-      </c>
-      <c r="D1036" t="s">
-        <v>1015</v>
-      </c>
-      <c r="G1036" s="11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="1037" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1037" t="s">
-        <v>1013</v>
-      </c>
-      <c r="B1037" t="s">
-        <v>1033</v>
-      </c>
-      <c r="C1037" t="s">
-        <v>1003</v>
-      </c>
-      <c r="D1037" t="s">
-        <v>1016</v>
-      </c>
-      <c r="G1037" s="11">
-        <v>3</v>
-      </c>
+      <c r="H1037" s="12"/>
     </row>
     <row r="1038" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1038" t="s">
@@ -26384,13 +26405,13 @@
         <v>1033</v>
       </c>
       <c r="C1038" t="s">
-        <v>1005</v>
+        <v>1000</v>
       </c>
       <c r="D1038" t="s">
-        <v>1017</v>
+        <v>10</v>
       </c>
       <c r="G1038" s="11">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1039" spans="1:8" x14ac:dyDescent="0.2">
@@ -26401,13 +26422,13 @@
         <v>1033</v>
       </c>
       <c r="C1039" t="s">
-        <v>1111</v>
+        <v>1001</v>
       </c>
       <c r="D1039" t="s">
-        <v>1112</v>
+        <v>1015</v>
       </c>
       <c r="G1039" s="11">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1040" spans="1:8" x14ac:dyDescent="0.2">
@@ -26418,13 +26439,13 @@
         <v>1033</v>
       </c>
       <c r="C1040" t="s">
-        <v>999</v>
+        <v>1003</v>
       </c>
       <c r="D1040" t="s">
-        <v>1385</v>
+        <v>1016</v>
       </c>
       <c r="G1040" s="11">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1041" spans="1:7" x14ac:dyDescent="0.2">
@@ -26435,16 +26456,13 @@
         <v>1033</v>
       </c>
       <c r="C1041" t="s">
-        <v>1107</v>
+        <v>1005</v>
       </c>
       <c r="D1041" t="s">
-        <v>1091</v>
-      </c>
-      <c r="E1041" t="s">
-        <v>86</v>
+        <v>1017</v>
       </c>
       <c r="G1041" s="11">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="1042" spans="1:7" x14ac:dyDescent="0.2">
@@ -26455,16 +26473,13 @@
         <v>1033</v>
       </c>
       <c r="C1042" t="s">
-        <v>1029</v>
+        <v>1111</v>
       </c>
       <c r="D1042" t="s">
-        <v>1046</v>
-      </c>
-      <c r="E1042" t="s">
-        <v>86</v>
+        <v>1112</v>
       </c>
       <c r="G1042" s="11">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1043" spans="1:7" x14ac:dyDescent="0.2">
@@ -26475,16 +26490,13 @@
         <v>1033</v>
       </c>
       <c r="C1043" t="s">
-        <v>1026</v>
+        <v>999</v>
       </c>
       <c r="D1043" t="s">
-        <v>1047</v>
-      </c>
-      <c r="E1043" t="s">
-        <v>86</v>
+        <v>1385</v>
       </c>
       <c r="G1043" s="11">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="1044" spans="1:7" x14ac:dyDescent="0.2">
@@ -26495,16 +26507,16 @@
         <v>1033</v>
       </c>
       <c r="C1044" t="s">
-        <v>1024</v>
+        <v>1107</v>
       </c>
       <c r="D1044" t="s">
-        <v>1048</v>
+        <v>1091</v>
       </c>
       <c r="E1044" t="s">
         <v>86</v>
       </c>
       <c r="G1044" s="11">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="1045" spans="1:7" x14ac:dyDescent="0.2">
@@ -26515,16 +26527,16 @@
         <v>1033</v>
       </c>
       <c r="C1045" t="s">
-        <v>1092</v>
+        <v>1029</v>
       </c>
       <c r="D1045" t="s">
-        <v>1102</v>
+        <v>1046</v>
       </c>
       <c r="E1045" t="s">
         <v>86</v>
       </c>
       <c r="G1045" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="1046" spans="1:7" x14ac:dyDescent="0.2">
@@ -26535,16 +26547,16 @@
         <v>1033</v>
       </c>
       <c r="C1046" t="s">
-        <v>1093</v>
+        <v>1026</v>
       </c>
       <c r="D1046" t="s">
-        <v>1103</v>
+        <v>1047</v>
       </c>
       <c r="E1046" t="s">
         <v>86</v>
       </c>
       <c r="G1046" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="1047" spans="1:7" x14ac:dyDescent="0.2">
@@ -26555,16 +26567,16 @@
         <v>1033</v>
       </c>
       <c r="C1047" t="s">
-        <v>1094</v>
+        <v>1024</v>
       </c>
       <c r="D1047" t="s">
-        <v>1105</v>
+        <v>1048</v>
       </c>
       <c r="E1047" t="s">
         <v>86</v>
       </c>
       <c r="G1047" s="11">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="1048" spans="1:7" x14ac:dyDescent="0.2">
@@ -26575,16 +26587,16 @@
         <v>1033</v>
       </c>
       <c r="C1048" t="s">
-        <v>1095</v>
+        <v>1092</v>
       </c>
       <c r="D1048" t="s">
-        <v>1104</v>
+        <v>1102</v>
       </c>
       <c r="E1048" t="s">
         <v>86</v>
       </c>
       <c r="G1048" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="1049" spans="1:7" x14ac:dyDescent="0.2">
@@ -26595,16 +26607,16 @@
         <v>1033</v>
       </c>
       <c r="C1049" t="s">
-        <v>1096</v>
+        <v>1093</v>
       </c>
       <c r="D1049" t="s">
-        <v>1106</v>
+        <v>1103</v>
       </c>
       <c r="E1049" t="s">
         <v>86</v>
       </c>
       <c r="G1049" s="11">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1050" spans="1:7" x14ac:dyDescent="0.2">
@@ -26612,16 +26624,19 @@
         <v>1013</v>
       </c>
       <c r="B1050" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="C1050" t="s">
-        <v>1000</v>
+        <v>1094</v>
       </c>
       <c r="D1050" t="s">
-        <v>10</v>
+        <v>1105</v>
+      </c>
+      <c r="E1050" t="s">
+        <v>86</v>
       </c>
       <c r="G1050" s="11">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="1051" spans="1:7" x14ac:dyDescent="0.2">
@@ -26629,16 +26644,19 @@
         <v>1013</v>
       </c>
       <c r="B1051" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="C1051" t="s">
-        <v>1001</v>
+        <v>1095</v>
       </c>
       <c r="D1051" t="s">
-        <v>1015</v>
+        <v>1104</v>
+      </c>
+      <c r="E1051" t="s">
+        <v>86</v>
       </c>
       <c r="G1051" s="11">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="1052" spans="1:7" x14ac:dyDescent="0.2">
@@ -26646,16 +26664,19 @@
         <v>1013</v>
       </c>
       <c r="B1052" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="C1052" t="s">
-        <v>1003</v>
+        <v>1096</v>
       </c>
       <c r="D1052" t="s">
-        <v>1016</v>
+        <v>1106</v>
+      </c>
+      <c r="E1052" t="s">
+        <v>86</v>
       </c>
       <c r="G1052" s="11">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="1053" spans="1:7" x14ac:dyDescent="0.2">
@@ -26666,13 +26687,13 @@
         <v>1034</v>
       </c>
       <c r="C1053" t="s">
-        <v>1005</v>
+        <v>1000</v>
       </c>
       <c r="D1053" t="s">
-        <v>1017</v>
+        <v>10</v>
       </c>
       <c r="G1053" s="11">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1054" spans="1:7" x14ac:dyDescent="0.2">
@@ -26683,13 +26704,13 @@
         <v>1034</v>
       </c>
       <c r="C1054" t="s">
-        <v>1111</v>
+        <v>1001</v>
       </c>
       <c r="D1054" t="s">
-        <v>1112</v>
+        <v>1015</v>
       </c>
       <c r="G1054" s="11">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1055" spans="1:7" x14ac:dyDescent="0.2">
@@ -26700,13 +26721,13 @@
         <v>1034</v>
       </c>
       <c r="C1055" t="s">
-        <v>999</v>
+        <v>1003</v>
       </c>
       <c r="D1055" t="s">
-        <v>1385</v>
+        <v>1016</v>
       </c>
       <c r="G1055" s="11">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1056" spans="1:7" x14ac:dyDescent="0.2">
@@ -26717,16 +26738,13 @@
         <v>1034</v>
       </c>
       <c r="C1056" t="s">
-        <v>1018</v>
+        <v>1005</v>
       </c>
       <c r="D1056" t="s">
-        <v>1041</v>
-      </c>
-      <c r="E1056" t="s">
-        <v>86</v>
+        <v>1017</v>
       </c>
       <c r="G1056" s="11">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="1057" spans="1:7" x14ac:dyDescent="0.2">
@@ -26737,16 +26755,13 @@
         <v>1034</v>
       </c>
       <c r="C1057" t="s">
-        <v>1020</v>
+        <v>1111</v>
       </c>
       <c r="D1057" t="s">
-        <v>1042</v>
-      </c>
-      <c r="E1057" t="s">
-        <v>86</v>
+        <v>1112</v>
       </c>
       <c r="G1057" s="11">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1058" spans="1:7" x14ac:dyDescent="0.2">
@@ -26757,16 +26772,13 @@
         <v>1034</v>
       </c>
       <c r="C1058" t="s">
-        <v>1022</v>
+        <v>999</v>
       </c>
       <c r="D1058" t="s">
-        <v>1043</v>
-      </c>
-      <c r="E1058" t="s">
-        <v>86</v>
+        <v>1385</v>
       </c>
       <c r="G1058" s="11">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="1059" spans="1:7" x14ac:dyDescent="0.2">
@@ -26777,16 +26789,16 @@
         <v>1034</v>
       </c>
       <c r="C1059" t="s">
-        <v>1026</v>
+        <v>1018</v>
       </c>
       <c r="D1059" t="s">
-        <v>1044</v>
+        <v>1041</v>
       </c>
       <c r="E1059" t="s">
         <v>86</v>
       </c>
       <c r="G1059" s="11">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="1060" spans="1:7" x14ac:dyDescent="0.2">
@@ -26797,16 +26809,16 @@
         <v>1034</v>
       </c>
       <c r="C1060" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="D1060" t="s">
-        <v>1045</v>
+        <v>1042</v>
       </c>
       <c r="E1060" t="s">
         <v>86</v>
       </c>
       <c r="G1060" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="1061" spans="1:7" x14ac:dyDescent="0.2">
@@ -26814,16 +26826,19 @@
         <v>1013</v>
       </c>
       <c r="B1061" t="s">
-        <v>1108</v>
+        <v>1034</v>
       </c>
       <c r="C1061" t="s">
-        <v>1000</v>
+        <v>1022</v>
       </c>
       <c r="D1061" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1061" s="2">
-        <v>1</v>
+        <v>1043</v>
+      </c>
+      <c r="E1061" t="s">
+        <v>86</v>
+      </c>
+      <c r="G1061" s="11">
+        <v>9</v>
       </c>
     </row>
     <row r="1062" spans="1:7" x14ac:dyDescent="0.2">
@@ -26831,16 +26846,19 @@
         <v>1013</v>
       </c>
       <c r="B1062" t="s">
-        <v>1108</v>
+        <v>1034</v>
       </c>
       <c r="C1062" t="s">
-        <v>1109</v>
+        <v>1026</v>
       </c>
       <c r="D1062" t="s">
-        <v>1110</v>
-      </c>
-      <c r="G1062" s="2">
-        <v>2</v>
+        <v>1044</v>
+      </c>
+      <c r="E1062" t="s">
+        <v>86</v>
+      </c>
+      <c r="G1062" s="11">
+        <v>10</v>
       </c>
     </row>
     <row r="1063" spans="1:7" x14ac:dyDescent="0.2">
@@ -26848,16 +26866,19 @@
         <v>1013</v>
       </c>
       <c r="B1063" t="s">
-        <v>1028</v>
+        <v>1034</v>
       </c>
       <c r="C1063" t="s">
-        <v>1000</v>
+        <v>1024</v>
       </c>
       <c r="D1063" t="s">
-        <v>10</v>
+        <v>1045</v>
+      </c>
+      <c r="E1063" t="s">
+        <v>86</v>
       </c>
       <c r="G1063" s="11">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="1064" spans="1:7" x14ac:dyDescent="0.2">
@@ -26865,16 +26886,16 @@
         <v>1013</v>
       </c>
       <c r="B1064" t="s">
-        <v>1028</v>
+        <v>1108</v>
       </c>
       <c r="C1064" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="D1064" t="s">
-        <v>1015</v>
-      </c>
-      <c r="G1064" s="11">
-        <v>2</v>
+        <v>10</v>
+      </c>
+      <c r="G1064" s="2">
+        <v>1</v>
       </c>
     </row>
     <row r="1065" spans="1:7" x14ac:dyDescent="0.2">
@@ -26882,16 +26903,16 @@
         <v>1013</v>
       </c>
       <c r="B1065" t="s">
-        <v>1028</v>
+        <v>1108</v>
       </c>
       <c r="C1065" t="s">
-        <v>1003</v>
+        <v>1109</v>
       </c>
       <c r="D1065" t="s">
-        <v>1016</v>
-      </c>
-      <c r="G1065" s="11">
-        <v>3</v>
+        <v>1110</v>
+      </c>
+      <c r="G1065" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="1066" spans="1:7" x14ac:dyDescent="0.2">
@@ -26902,13 +26923,13 @@
         <v>1028</v>
       </c>
       <c r="C1066" t="s">
-        <v>1005</v>
+        <v>1000</v>
       </c>
       <c r="D1066" t="s">
-        <v>1017</v>
+        <v>10</v>
       </c>
       <c r="G1066" s="11">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1067" spans="1:7" x14ac:dyDescent="0.2">
@@ -26919,13 +26940,13 @@
         <v>1028</v>
       </c>
       <c r="C1067" t="s">
-        <v>1111</v>
+        <v>1001</v>
       </c>
       <c r="D1067" t="s">
-        <v>1112</v>
+        <v>1015</v>
       </c>
       <c r="G1067" s="11">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1068" spans="1:7" x14ac:dyDescent="0.2">
@@ -26936,13 +26957,13 @@
         <v>1028</v>
       </c>
       <c r="C1068" t="s">
-        <v>999</v>
+        <v>1003</v>
       </c>
       <c r="D1068" t="s">
-        <v>1385</v>
+        <v>1016</v>
       </c>
       <c r="G1068" s="11">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1069" spans="1:7" x14ac:dyDescent="0.2">
@@ -26953,16 +26974,13 @@
         <v>1028</v>
       </c>
       <c r="C1069" t="s">
-        <v>1107</v>
+        <v>1005</v>
       </c>
       <c r="D1069" t="s">
-        <v>1090</v>
-      </c>
-      <c r="E1069" t="s">
-        <v>86</v>
+        <v>1017</v>
       </c>
       <c r="G1069" s="11">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="1070" spans="1:7" x14ac:dyDescent="0.2">
@@ -26973,16 +26991,13 @@
         <v>1028</v>
       </c>
       <c r="C1070" t="s">
-        <v>1029</v>
+        <v>1111</v>
       </c>
       <c r="D1070" t="s">
-        <v>1030</v>
-      </c>
-      <c r="E1070" t="s">
-        <v>86</v>
+        <v>1112</v>
       </c>
       <c r="G1070" s="11">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1071" spans="1:7" x14ac:dyDescent="0.2">
@@ -26993,16 +27008,13 @@
         <v>1028</v>
       </c>
       <c r="C1071" t="s">
-        <v>1026</v>
+        <v>999</v>
       </c>
       <c r="D1071" t="s">
-        <v>1031</v>
-      </c>
-      <c r="E1071" t="s">
-        <v>86</v>
+        <v>1385</v>
       </c>
       <c r="G1071" s="11">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="1072" spans="1:7" x14ac:dyDescent="0.2">
@@ -27013,16 +27025,16 @@
         <v>1028</v>
       </c>
       <c r="C1072" t="s">
-        <v>1024</v>
+        <v>1107</v>
       </c>
       <c r="D1072" t="s">
-        <v>1032</v>
+        <v>1090</v>
       </c>
       <c r="E1072" t="s">
         <v>86</v>
       </c>
       <c r="G1072" s="11">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="1073" spans="1:7" x14ac:dyDescent="0.2">
@@ -27033,16 +27045,16 @@
         <v>1028</v>
       </c>
       <c r="C1073" t="s">
-        <v>1092</v>
+        <v>1029</v>
       </c>
       <c r="D1073" t="s">
-        <v>1097</v>
+        <v>1030</v>
       </c>
       <c r="E1073" t="s">
         <v>86</v>
       </c>
       <c r="G1073" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="1074" spans="1:7" x14ac:dyDescent="0.2">
@@ -27053,16 +27065,16 @@
         <v>1028</v>
       </c>
       <c r="C1074" t="s">
-        <v>1093</v>
+        <v>1026</v>
       </c>
       <c r="D1074" t="s">
-        <v>1098</v>
+        <v>1031</v>
       </c>
       <c r="E1074" t="s">
         <v>86</v>
       </c>
       <c r="G1074" s="11">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="1075" spans="1:7" x14ac:dyDescent="0.2">
@@ -27073,16 +27085,16 @@
         <v>1028</v>
       </c>
       <c r="C1075" t="s">
-        <v>1094</v>
+        <v>1024</v>
       </c>
       <c r="D1075" t="s">
-        <v>1099</v>
+        <v>1032</v>
       </c>
       <c r="E1075" t="s">
         <v>86</v>
       </c>
       <c r="G1075" s="11">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="1076" spans="1:7" x14ac:dyDescent="0.2">
@@ -27093,16 +27105,16 @@
         <v>1028</v>
       </c>
       <c r="C1076" t="s">
-        <v>1095</v>
+        <v>1092</v>
       </c>
       <c r="D1076" t="s">
-        <v>1100</v>
+        <v>1097</v>
       </c>
       <c r="E1076" t="s">
         <v>86</v>
       </c>
       <c r="G1076" s="11">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="1077" spans="1:7" x14ac:dyDescent="0.2">
@@ -27113,16 +27125,16 @@
         <v>1028</v>
       </c>
       <c r="C1077" t="s">
-        <v>1096</v>
+        <v>1093</v>
       </c>
       <c r="D1077" t="s">
-        <v>1101</v>
+        <v>1098</v>
       </c>
       <c r="E1077" t="s">
         <v>86</v>
       </c>
       <c r="G1077" s="11">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="1078" spans="1:7" x14ac:dyDescent="0.2">
@@ -27130,16 +27142,19 @@
         <v>1013</v>
       </c>
       <c r="B1078" t="s">
-        <v>1014</v>
+        <v>1028</v>
       </c>
       <c r="C1078" t="s">
-        <v>1000</v>
+        <v>1094</v>
       </c>
       <c r="D1078" t="s">
-        <v>10</v>
+        <v>1099</v>
+      </c>
+      <c r="E1078" t="s">
+        <v>86</v>
       </c>
       <c r="G1078" s="11">
-        <v>1</v>
+        <v>13</v>
       </c>
     </row>
     <row r="1079" spans="1:7" x14ac:dyDescent="0.2">
@@ -27147,16 +27162,19 @@
         <v>1013</v>
       </c>
       <c r="B1079" t="s">
-        <v>1014</v>
+        <v>1028</v>
       </c>
       <c r="C1079" t="s">
-        <v>1001</v>
+        <v>1095</v>
       </c>
       <c r="D1079" t="s">
-        <v>1015</v>
+        <v>1100</v>
+      </c>
+      <c r="E1079" t="s">
+        <v>86</v>
       </c>
       <c r="G1079" s="11">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="1080" spans="1:7" x14ac:dyDescent="0.2">
@@ -27164,16 +27182,19 @@
         <v>1013</v>
       </c>
       <c r="B1080" t="s">
-        <v>1014</v>
+        <v>1028</v>
       </c>
       <c r="C1080" t="s">
-        <v>1003</v>
+        <v>1096</v>
       </c>
       <c r="D1080" t="s">
-        <v>1016</v>
+        <v>1101</v>
+      </c>
+      <c r="E1080" t="s">
+        <v>86</v>
       </c>
       <c r="G1080" s="11">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="1081" spans="1:7" x14ac:dyDescent="0.2">
@@ -27184,13 +27205,13 @@
         <v>1014</v>
       </c>
       <c r="C1081" t="s">
-        <v>1005</v>
+        <v>1000</v>
       </c>
       <c r="D1081" t="s">
-        <v>1017</v>
+        <v>10</v>
       </c>
       <c r="G1081" s="11">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="1082" spans="1:7" x14ac:dyDescent="0.2">
@@ -27201,13 +27222,13 @@
         <v>1014</v>
       </c>
       <c r="C1082" t="s">
-        <v>1111</v>
+        <v>1001</v>
       </c>
       <c r="D1082" t="s">
-        <v>1112</v>
+        <v>1015</v>
       </c>
       <c r="G1082" s="11">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="1083" spans="1:7" x14ac:dyDescent="0.2">
@@ -27218,13 +27239,13 @@
         <v>1014</v>
       </c>
       <c r="C1083" t="s">
-        <v>999</v>
+        <v>1003</v>
       </c>
       <c r="D1083" t="s">
-        <v>1385</v>
+        <v>1016</v>
       </c>
       <c r="G1083" s="11">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="1084" spans="1:7" x14ac:dyDescent="0.2">
@@ -27235,16 +27256,13 @@
         <v>1014</v>
       </c>
       <c r="C1084" t="s">
-        <v>1018</v>
+        <v>1005</v>
       </c>
       <c r="D1084" t="s">
-        <v>1019</v>
-      </c>
-      <c r="E1084" t="s">
-        <v>86</v>
+        <v>1017</v>
       </c>
       <c r="G1084" s="11">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="1085" spans="1:7" x14ac:dyDescent="0.2">
@@ -27255,16 +27273,13 @@
         <v>1014</v>
       </c>
       <c r="C1085" t="s">
-        <v>1020</v>
+        <v>1111</v>
       </c>
       <c r="D1085" t="s">
-        <v>1021</v>
-      </c>
-      <c r="E1085" t="s">
-        <v>86</v>
+        <v>1112</v>
       </c>
       <c r="G1085" s="11">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="1086" spans="1:7" x14ac:dyDescent="0.2">
@@ -27275,16 +27290,13 @@
         <v>1014</v>
       </c>
       <c r="C1086" t="s">
-        <v>1022</v>
+        <v>999</v>
       </c>
       <c r="D1086" t="s">
-        <v>1023</v>
-      </c>
-      <c r="E1086" t="s">
-        <v>86</v>
+        <v>1385</v>
       </c>
       <c r="G1086" s="11">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="1087" spans="1:7" x14ac:dyDescent="0.2">
@@ -27295,16 +27307,16 @@
         <v>1014</v>
       </c>
       <c r="C1087" t="s">
-        <v>1024</v>
+        <v>1018</v>
       </c>
       <c r="D1087" t="s">
-        <v>1025</v>
+        <v>1019</v>
       </c>
       <c r="E1087" t="s">
         <v>86</v>
       </c>
       <c r="G1087" s="11">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="1088" spans="1:7" x14ac:dyDescent="0.2">
@@ -27315,28 +27327,80 @@
         <v>1014</v>
       </c>
       <c r="C1088" t="s">
-        <v>1026</v>
+        <v>1020</v>
       </c>
       <c r="D1088" t="s">
-        <v>1027</v>
+        <v>1021</v>
       </c>
       <c r="E1088" t="s">
         <v>86</v>
       </c>
       <c r="G1088" s="11">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1089" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B1089" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C1089" t="s">
+        <v>1022</v>
+      </c>
+      <c r="D1089" t="s">
+        <v>1023</v>
+      </c>
+      <c r="E1089" t="s">
+        <v>86</v>
+      </c>
+      <c r="G1089" s="11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1090" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B1090" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C1090" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D1090" t="s">
+        <v>1025</v>
+      </c>
+      <c r="E1090" t="s">
+        <v>86</v>
+      </c>
+      <c r="G1090" s="11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1091" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B1091" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C1091" t="s">
+        <v>1026</v>
+      </c>
+      <c r="D1091" t="s">
+        <v>1027</v>
+      </c>
+      <c r="E1091" t="s">
+        <v>86</v>
+      </c>
+      <c r="G1091" s="11">
         <v>11</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1088" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H1088">
-      <sortCondition ref="A2:A1088"/>
-      <sortCondition ref="H2:H1088"/>
-      <sortCondition ref="F2:F1088"/>
-      <sortCondition ref="B2:B1088"/>
-      <sortCondition ref="G2:G1088"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:H1091" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>